<commit_message>
Consolidate Discovery Workbook against old DBC worksheets, add 5 non-overlapping questions
Cross-checked Consumer and Organization Discovery tabs against three older
DBC-specific discovery documents. No overlapping questions needed rewording,
they were already near-duplicates in W04/W03 phrasing. Added the 5 genuinely
new questions that existed only in the old worksheets: 4 to Consumer
Discovery, 1 to Organization Discovery.
</commit_message>
<xml_diff>
--- a/templates/Discovery_Workbook_Template.xlsx
+++ b/templates/Discovery_Workbook_Template.xlsx
@@ -1059,7 +1059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1313,6 +1313,21 @@
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Sales, engagement, customer behavior, anything. Be honest about what you have versus what you wish you had.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>What does "improving the business" mean to you, specifically?</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Not the general goal. The concrete version: which numbers move, which problems disappear, what does better actually look like.</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1671,6 +1686,66 @@
         </is>
       </c>
     </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>Are they buying for themselves or for someone else?</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Is this customer the end user, or are they buying, choosing, or approving on someone else's behalf?</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>Do they come to you with a specific need, or as part of a larger project?</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Is this a standalone purchase, or one piece of something bigger they are trying to accomplish?</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>How knowledgeable are they about the category when they find you?</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Are they new to this and learning as they go, or already fluent and comparing options with expertise?</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>How much do they typically spend, and how often do they order?</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>What does a normal transaction look like, and what does normal frequency look like over a year?</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A5:B5"/>

</xml_diff>